<commit_message>
Sushi Restaurant Business Plan Kit EN · F2 cerrada: revisión adversarial (0 B · 2 M · 14 m, todos arreglados), 4 entregables regenerados (G1-G9 TODO VERDE, canon 4/4 IGUAL), F2-NOTAS y REVISION-FINAL
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/sushi-restaurant-business-plan/sushi-fish-rice-costing-calculator.xlsx
+++ b/astro-site/public/dl/sushi-restaurant-business-plan/sushi-fish-rice-costing-calculator.xlsx
@@ -612,7 +612,7 @@
     <row r="3" ht="64" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>FIXED NOTICE. Parasite destruction (FDA Food Code 2022, 3-402.11): fish served raw or undercooked is frozen at −4 °F or below for 168 hours (7 days), or at −31 °F until solid and held 15 hours, or at −31 °F until solid and held 24 hours at −4 °F. Tuna species and feed-raised aquaculture fish are exempt only with a written statement from the supplier or the farm. Keep the records 90 days (3-402.12). Your county's rules may be stricter. The cleaning minutes (25) have no source: time it.</t>
+          <t>FIXED NOTICE. Parasite destruction (FDA Food Code 2022, 3-402.11): fish served raw or undercooked is frozen at −4 °F or below for 168 hours (7 days), or at −31 °F until solid and held 15 hours, or at −31 °F until solid and held 24 hours at −4 °F. Tuna species are exempt; feed-raised aquaculture fish only with a written statement from the supplier or the farm. Keep the records 90 days (3-402.12). Your county's rules may be stricter. The cleaning minutes (25) have no source: time it.</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Tuna (Thunnus species) and feed-raised aquaculture fish such as farmed salmon are exempt only with a written statement from the supplier or the farm. File it and ask again if the source changes.</t>
+          <t>Tuna (Thunnus species) is exempt; feed-raised aquaculture fish such as farmed salmon is exempt only with a written statement from the supplier or the farm. Keep the tuna invoice that names the species, file the statement and ask again if the source changes.</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>50 lb bag $51.99 = $1.04/lb, webstaurantstore.com, Oct 2026; medium grain $1.24-1.28/lb.</t>
+          <t>50 lb bag $51.99 = $1.04/lb, webstaurantstore.com, Oct 2026; other medium-grain brands $1.24-1.28/lb.</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
     <row r="12" ht="105" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>4. Parasite destruction (FDA Food Code 2022, 3-402.11). Fish served raw or undercooked is frozen at −4 °F or below for 168 hours (7 days), or at −31 °F until solid and held 15 hours, or at −31 °F until solid and held 24 hours at −4 °F. Tuna species and feed-raised aquaculture fish such as farmed salmon are exempt only with a written statement from the supplier or the farm. If the fish arrives frozen, keep the supplier's written agreement or statement for every lot, showing the freezing time and temperature. Keep the records 90 days (3-402.12). "Sushi-grade" has no legal definition: a supplier label is no substitute for the freezing records or the written statement. The dropdown on the sheet is a reminder only: it changes no figure.</t>
+          <t>4. Parasite destruction (FDA Food Code 2022, 3-402.11). Fish served raw or undercooked is frozen at −4 °F or below for 168 hours (7 days), or at −31 °F until solid and held 15 hours, or at −31 °F until solid and held 24 hours at −4 °F. Tuna species and feed-raised aquaculture fish such as farmed salmon are exempt; the farmed fish only with a written statement from the supplier or the farm, and the kit also files the tuna invoice that names the species. If the fish arrives frozen, keep the supplier's written agreement or statement for every lot, showing the freezing time and temperature. Keep the records 90 days (3-402.12). "Sushi-grade" has no legal definition: a supplier label is no substitute for the freezing records or the written statement. The dropdown on the sheet is a reminder only: it changes no figure.</t>
         </is>
       </c>
     </row>

</xml_diff>